<commit_message>
contracts, AOs, materials, issues, invoice history importers + pages; templates without cell comments (exceljs-readable) and example-row skipping
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/01_الهيكل_التنظيمي.xlsx
+++ b/apps/web/public/templates/01_الهيكل_التنظيمي.xlsx
@@ -230,51 +230,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>المنظومة</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>كود قصير فريد مثل PR-DELTA</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>المنظومة</author>
-  </authors>
-  <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>من شيت رئاسات القطاعات</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>المنظومة</author>
-  </authors>
-  <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>اختياري — بيتربط بالمستخدم</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -611,7 +566,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -682,7 +636,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -769,7 +722,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -989,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1096,6 +1048,37 @@
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>• نسخة القالب: 1.0 — لو القالب قديم السيستم هيطلب تنزيل النسخة الجديدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>شرح الأعمدة</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>• [رئاسات القطاعات] كود الرئاسة: كود قصير فريد مثل PR-DELTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>• [القطاعات] كود الرئاسة: من شيت رئاسات القطاعات</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>• [الإدارات العامة] إيميل المدير العام: اختياري — بيتربط بالمستخدم</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1137,6 +1120,18 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>examples</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"رئاسات القطاعات": [["PR-DELTA", "رئاسة قطاعات الدلتا والقناة"]], "القطاعات": [["S-EAST", "PR-DELTA", "المنطقة الشرقية"]], "الإدارات العامة": [["G-SINAI", "S-EAST", "الإدارة العامة لمناطق شمال سيناء", "gm.sinai@te.eg"]], "الشئون الفنية": [["TA-EAST", "S-EAST", "الشئون الفنية — المنطقة الشرقية"]], "الإدارات المختصة": [["D-ARISH", "G-SINAI", "إدارة تنفيذ العريش"]], "السنترالات": [["C-RABAA", "D-ARISH", "سنترال رابعة"]]}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
copy: formal Modern Standard Arabic with PMI/ERP terminology across UI, errors, emails, templates and seed (idempotent rename of seeded labels)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/01_الهيكل_التنظيمي.xlsx
+++ b/apps/web/public/templates/01_الهيكل_التنظيمي.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>إيميل المدير العام</t>
+          <t>البريد الإلكتروني للمدير العام</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>قالب الهيكل التنظيمي</t>
+          <t>نموذج الهيكل التنظيمي</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>مين بيرفعه: مدير النظام (Admin).</t>
+          <t>الجهة المسؤولة عن الرفع: مدير النظام (Admin).</t>
         </is>
       </c>
     </row>
@@ -974,28 +974,28 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>قواعد الملء</t>
+          <t>قواعد تعبئة البيانات</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>• ابدأ من الشيت الأول للأخير — كل مستوى بيشاور على كود المستوى اللي فوقه.</t>
+          <t>• يرجى التعبئة من ورقة العمل الأولى حتى الأخيرة — يُشار في كل مستوى إلى كود المستوى الأعلى منه.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>• الكود فريد ومش بيتغير بعد الرفع (الاسم ممكن يتعدل).</t>
+          <t>• الكود فريد ولا يتغير بعد الرفع (يمكن تعديل الاسم).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>• لو الرفع لكيان موجود بنفس الكود، السيستم بيحدّث الاسم بس.</t>
+          <t>• عند رفع كيان مسجل بالكود نفسه، تُحدِّث المنظومة الاسم فقط.</t>
         </is>
       </c>
     </row>
@@ -1005,49 +1005,49 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>قواعد عامة لكل القوالب</t>
+          <t>قواعد عامة لجميع النماذج</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>• ما تغيّرش أسماء الشيتات ولا ترتيب الأعمدة ولا الصف التاني (اسم العمود التقني).</t>
+          <t>• لا يجوز تغيير أسماء أوراق العمل أو ترتيب الأعمدة أو الصف الثاني (الاسم التقني للعمود).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>• العمود اللي عليه * إلزامي. الأعمدة اللي فيها قائمة لازم تختار منها.</t>
+          <t>• العمود المميز بعلامة * إلزامي، ويجب الاختيار من القائمة في الأعمدة التي تتضمن قائمة اختيار.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>• الصفوف الرمادي أمثلة — امسحها قبل الرفع.</t>
+          <t>• الصفوف الرمادية أمثلة توضيحية — يرجى حذفها قبل الرفع.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>• الأرقام من غير فواصل أو عملة. التواريخ يوم/شهر/سنة.</t>
+          <t>• تُدخل الأرقام دون فواصل أو رمز عملة، والتواريخ بصيغة يوم/شهر/سنة.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>• عند الرفع السيستم بيعرض معاينة بكل صف وأخطاؤه قبل الحفظ — مفيش حاجة بتتحفظ قبل ما توافق.</t>
+          <t>• عند الرفع تعرض المنظومة نتيجة المراجعة لكل صف وأخطاءه قبل الحفظ — ولا يُحفظ أي سجل قبل «اعتماد الاستيراد».</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>• نسخة القالب: 1.0 — لو القالب قديم السيستم هيطلب تنزيل النسخة الجديدة.</t>
+          <t>• إصدار النموذج: 1.0 — إذا كان النموذج قديماً ستطلب المنظومة تحميل الإصدار الأحدث.</t>
         </is>
       </c>
     </row>
@@ -1057,28 +1057,28 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>شرح الأعمدة</t>
+          <t>إيضاح الأعمدة</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>• [رئاسات القطاعات] كود الرئاسة: كود قصير فريد مثل PR-DELTA</t>
+          <t>• [رئاسات القطاعات] كود الرئاسة: كود مختصر فريد، مثال: PR-DELTA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>• [القطاعات] كود الرئاسة: من شيت رئاسات القطاعات</t>
+          <t>• [القطاعات] كود الرئاسة: من ورقة عمل رئاسات القطاعات</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>• [الإدارات العامة] إيميل المدير العام: اختياري — بيتربط بالمستخدم</t>
+          <t>• [الإدارات العامة] البريد الإلكتروني للمدير العام: اختياري — يُربط بحساب المستخدم</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
templates: mark example rows with 'مثال —' so real rows (e.g. BOQ headings) can never match and be skipped
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/01_الهيكل_التنظيمي.xlsx
+++ b/apps/web/public/templates/01_الهيكل_التنظيمي.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>رئاسة قطاعات الدلتا والقناة</t>
+          <t>مثال — رئاسة قطاعات الدلتا والقناة</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>المنطقة الشرقية</t>
+          <t>مثال — المنطقة الشرقية</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>الإدارة العامة لمناطق شمال سيناء</t>
+          <t>مثال — الإدارة العامة لمناطق شمال سيناء</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>الشئون الفنية — المنطقة الشرقية</t>
+          <t>مثال — الشئون الفنية — المنطقة الشرقية</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>إدارة تنفيذ العريش</t>
+          <t>مثال — إدارة تنفيذ العريش</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>سنترال رابعة</t>
+          <t>مثال — سنترال رابعة</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"رئاسات القطاعات": [["PR-DELTA", "رئاسة قطاعات الدلتا والقناة"]], "القطاعات": [["S-EAST", "PR-DELTA", "المنطقة الشرقية"]], "الإدارات العامة": [["G-SINAI", "S-EAST", "الإدارة العامة لمناطق شمال سيناء", "gm.sinai@te.eg"]], "الشئون الفنية": [["TA-EAST", "S-EAST", "الشئون الفنية — المنطقة الشرقية"]], "الإدارات المختصة": [["D-ARISH", "G-SINAI", "إدارة تنفيذ العريش"]], "السنترالات": [["C-RABAA", "D-ARISH", "سنترال رابعة"]]}</t>
+          <t>{"رئاسات القطاعات": [["PR-DELTA", "مثال — رئاسة قطاعات الدلتا والقناة"]], "القطاعات": [["S-EAST", "PR-DELTA", "مثال — المنطقة الشرقية"]], "الإدارات العامة": [["G-SINAI", "S-EAST", "مثال — الإدارة العامة لمناطق شمال سيناء", "gm.sinai@te.eg"]], "الشئون الفنية": [["TA-EAST", "S-EAST", "مثال — الشئون الفنية — المنطقة الشرقية"]], "الإدارات المختصة": [["D-ARISH", "G-SINAI", "مثال — إدارة تنفيذ العريش"]], "السنترالات": [["C-RABAA", "D-ARISH", "مثال — سنترال رابعة"]]}</t>
         </is>
       </c>
     </row>

</xml_diff>